<commit_message>
[FINANCE] Make IRR/NPV formulas locale-independent
</commit_message>
<xml_diff>
--- a/models/financial/financial_model_crowdfunding.xlsx
+++ b/models/financial/financial_model_crowdfunding.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AdelinePruvost\Documents\circular-energy-fund\models\financial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09F306A1-C111-40DF-B2F6-AEC5C0FB93E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965E7DCA-7EB9-4991-857A-6488062F55E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D264A57A-F8FE-4DF8-A1A7-B185DC2A0E30}"/>
   </bookViews>
@@ -19,6 +19,9 @@
     <sheet name="CAPEX" sheetId="2" r:id="rId4"/>
     <sheet name="Ricavi" sheetId="1" r:id="rId5"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId6"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Fonte</t>
   </si>
@@ -79,12 +82,30 @@
   </si>
   <si>
     <t>Netto</t>
+  </si>
+  <si>
+    <t>Tasso di sconto</t>
+  </si>
+  <si>
+    <t>Cumulato</t>
+  </si>
+  <si>
+    <t>ROI</t>
+  </si>
+  <si>
+    <t>IRR</t>
+  </si>
+  <si>
+    <t>NPV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -122,9 +143,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -140,6 +164,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Assumptions"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -459,16 +496,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E55BE27-92FE-47F5-9B77-15FAB5E6A743}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -480,6 +518,435 @@
       </c>
       <c r="D1" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="E1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>500000</v>
+      </c>
+      <c r="D2">
+        <f>B2-C2</f>
+        <v>-500000</v>
+      </c>
+      <c r="E2">
+        <f>SUM(D$2:D2)</f>
+        <v>-500000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>70000</v>
+      </c>
+      <c r="C3">
+        <v>10000</v>
+      </c>
+      <c r="D3">
+        <f>B3-C3</f>
+        <v>60000</v>
+      </c>
+      <c r="E3">
+        <f>SUM(D$2:D3)</f>
+        <v>-440000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>70000</v>
+      </c>
+      <c r="C4">
+        <v>10000</v>
+      </c>
+      <c r="D4">
+        <f>B4-C4</f>
+        <v>60000</v>
+      </c>
+      <c r="E4">
+        <f>SUM(D$2:D4)</f>
+        <v>-380000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>70000</v>
+      </c>
+      <c r="C5">
+        <v>10000</v>
+      </c>
+      <c r="D5">
+        <f>B5-C5</f>
+        <v>60000</v>
+      </c>
+      <c r="E5">
+        <f>SUM(D$2:D5)</f>
+        <v>-320000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>70000</v>
+      </c>
+      <c r="C6">
+        <v>10000</v>
+      </c>
+      <c r="D6">
+        <f>B6-C6</f>
+        <v>60000</v>
+      </c>
+      <c r="E6">
+        <f>SUM(D$2:D6)</f>
+        <v>-260000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>70000</v>
+      </c>
+      <c r="C7">
+        <v>10000</v>
+      </c>
+      <c r="D7">
+        <f>B7-C7</f>
+        <v>60000</v>
+      </c>
+      <c r="E7">
+        <f>SUM(D$2:D7)</f>
+        <v>-200000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>70000</v>
+      </c>
+      <c r="C8">
+        <v>10000</v>
+      </c>
+      <c r="D8">
+        <f>B8-C8</f>
+        <v>60000</v>
+      </c>
+      <c r="E8">
+        <f>SUM(D$2:D8)</f>
+        <v>-140000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>70000</v>
+      </c>
+      <c r="C9">
+        <v>10000</v>
+      </c>
+      <c r="D9">
+        <f>B9-C9</f>
+        <v>60000</v>
+      </c>
+      <c r="E9">
+        <f>SUM(D$2:D9)</f>
+        <v>-80000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>70000</v>
+      </c>
+      <c r="C10">
+        <v>10000</v>
+      </c>
+      <c r="D10">
+        <f>B10-C10</f>
+        <v>60000</v>
+      </c>
+      <c r="E10">
+        <f>SUM(D$2:D10)</f>
+        <v>-20000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>70000</v>
+      </c>
+      <c r="C11">
+        <v>10000</v>
+      </c>
+      <c r="D11">
+        <f>B11-C11</f>
+        <v>60000</v>
+      </c>
+      <c r="E11">
+        <f>SUM(D$2:D11)</f>
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>70000</v>
+      </c>
+      <c r="C12">
+        <v>10000</v>
+      </c>
+      <c r="D12">
+        <f>B12-C12</f>
+        <v>60000</v>
+      </c>
+      <c r="E12">
+        <f>SUM(D$2:D12)</f>
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>70000</v>
+      </c>
+      <c r="C13">
+        <v>10000</v>
+      </c>
+      <c r="D13">
+        <f>B13-C13</f>
+        <v>60000</v>
+      </c>
+      <c r="E13">
+        <f>SUM(D$2:D13)</f>
+        <v>160000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>70000</v>
+      </c>
+      <c r="C14">
+        <v>10000</v>
+      </c>
+      <c r="D14">
+        <f>B14-C14</f>
+        <v>60000</v>
+      </c>
+      <c r="E14">
+        <f>SUM(D$2:D14)</f>
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>70000</v>
+      </c>
+      <c r="C15">
+        <v>10000</v>
+      </c>
+      <c r="D15">
+        <f>B15-C15</f>
+        <v>60000</v>
+      </c>
+      <c r="E15">
+        <f>SUM(D$2:D15)</f>
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>70000</v>
+      </c>
+      <c r="C16">
+        <v>10000</v>
+      </c>
+      <c r="D16">
+        <f>B16-C16</f>
+        <v>60000</v>
+      </c>
+      <c r="E16">
+        <f>SUM(D$2:D16)</f>
+        <v>340000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>70000</v>
+      </c>
+      <c r="C17">
+        <v>10000</v>
+      </c>
+      <c r="D17">
+        <f>B17-C17</f>
+        <v>60000</v>
+      </c>
+      <c r="E17">
+        <f>SUM(D$2:D17)</f>
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>70000</v>
+      </c>
+      <c r="C18">
+        <v>10000</v>
+      </c>
+      <c r="D18">
+        <f>B18-C18</f>
+        <v>60000</v>
+      </c>
+      <c r="E18">
+        <f>SUM(D$2:D18)</f>
+        <v>460000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>70000</v>
+      </c>
+      <c r="C19">
+        <v>10000</v>
+      </c>
+      <c r="D19">
+        <f>B19-C19</f>
+        <v>60000</v>
+      </c>
+      <c r="E19">
+        <f>SUM(D$2:D19)</f>
+        <v>520000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>70000</v>
+      </c>
+      <c r="C20">
+        <v>10000</v>
+      </c>
+      <c r="D20">
+        <f>B20-C20</f>
+        <v>60000</v>
+      </c>
+      <c r="E20">
+        <f>SUM(D$2:D20)</f>
+        <v>580000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>70000</v>
+      </c>
+      <c r="C21">
+        <v>10000</v>
+      </c>
+      <c r="D21">
+        <f>B21-C21</f>
+        <v>60000</v>
+      </c>
+      <c r="E21">
+        <f>SUM(D$2:D21)</f>
+        <v>640000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>70000</v>
+      </c>
+      <c r="C22">
+        <v>10000</v>
+      </c>
+      <c r="D22">
+        <f>B22-C22</f>
+        <v>60000</v>
+      </c>
+      <c r="E22">
+        <f>SUM(D$2:D22)</f>
+        <v>700000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="3">
+        <f>IRR(D2:D22)</f>
+        <v>0.10315614602932954</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="4" t="e">
+        <f>NPV([1]Assumptions!B2,D3:D22)+D2</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26">
+        <f>(SUM(B2:B22)-SUM(C2:C22))/SUM(C2:C22)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -511,7 +978,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1CE410-6A17-4169-858C-950C42088566}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
@@ -528,6 +995,14 @@
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[DASHBOARD] Add automatic KPI dashboard
</commit_message>
<xml_diff>
--- a/models/financial/financial_model_crowdfunding.xlsx
+++ b/models/financial/financial_model_crowdfunding.xlsx
@@ -8,20 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AdelinePruvost\Documents\circular-energy-fund\models\financial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965E7DCA-7EB9-4991-857A-6488062F55E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91F4C12-D612-43AA-9BA8-A042E68E850B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D264A57A-F8FE-4DF8-A1A7-B185DC2A0E30}"/>
+    <workbookView xWindow="0" yWindow="240" windowWidth="17280" windowHeight="8880" xr2:uid="{D264A57A-F8FE-4DF8-A1A7-B185DC2A0E30}"/>
   </bookViews>
   <sheets>
-    <sheet name="Cashflow" sheetId="5" r:id="rId1"/>
-    <sheet name="OPEX" sheetId="4" r:id="rId2"/>
-    <sheet name="Assunzioni" sheetId="3" r:id="rId3"/>
-    <sheet name="CAPEX" sheetId="2" r:id="rId4"/>
-    <sheet name="Ricavi" sheetId="1" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="6" r:id="rId1"/>
+    <sheet name="Cashflow" sheetId="5" r:id="rId2"/>
+    <sheet name="OPEX" sheetId="4" r:id="rId3"/>
+    <sheet name="Assunzioni" sheetId="3" r:id="rId4"/>
+    <sheet name="CAPEX" sheetId="2" r:id="rId5"/>
+    <sheet name="Ricavi" sheetId="1" r:id="rId6"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId6"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Fonte</t>
   </si>
@@ -97,6 +95,15 @@
   </si>
   <si>
     <t>NPV</t>
+  </si>
+  <si>
+    <t>Dashboard KPI – Fondo Energetico Circolare</t>
+  </si>
+  <si>
+    <t>CAPEX Totale</t>
+  </si>
+  <si>
+    <t>Cashflow Finale</t>
   </si>
 </sst>
 </file>
@@ -104,9 +111,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="8" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="_-[$€-2]\ * #,##0.00_-;\-[$€-2]\ * #,##0.00_-;_-[$€-2]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,16 +129,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="43"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -139,19 +167,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -164,19 +215,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Assumptions"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -495,12 +533,83 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33298941-3A45-4CC1-A16E-D377190500EE}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="9">
+        <f>Cashflow!B24</f>
+        <v>0.10315614602932954</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="10">
+        <f>Cashflow!B25</f>
+        <v>188195.27311391488</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="9">
+        <f>Cashflow!B26</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="10">
+        <f>SUM(CAPEX!B:B)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="10">
+        <f>MAX(Cashflow!E:E)</f>
+        <v>700000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E55BE27-92FE-47F5-9B77-15FAB5E6A743}">
   <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -534,7 +643,7 @@
         <v>500000</v>
       </c>
       <c r="D2">
-        <f>B2-C2</f>
+        <f t="shared" ref="D2:D22" si="0">B2-C2</f>
         <v>-500000</v>
       </c>
       <c r="E2">
@@ -553,7 +662,7 @@
         <v>10000</v>
       </c>
       <c r="D3">
-        <f>B3-C3</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E3">
@@ -572,7 +681,7 @@
         <v>10000</v>
       </c>
       <c r="D4">
-        <f>B4-C4</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E4">
@@ -591,7 +700,7 @@
         <v>10000</v>
       </c>
       <c r="D5">
-        <f>B5-C5</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E5">
@@ -610,7 +719,7 @@
         <v>10000</v>
       </c>
       <c r="D6">
-        <f>B6-C6</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E6">
@@ -629,7 +738,7 @@
         <v>10000</v>
       </c>
       <c r="D7">
-        <f>B7-C7</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E7">
@@ -648,7 +757,7 @@
         <v>10000</v>
       </c>
       <c r="D8">
-        <f>B8-C8</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E8">
@@ -667,7 +776,7 @@
         <v>10000</v>
       </c>
       <c r="D9">
-        <f>B9-C9</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E9">
@@ -686,7 +795,7 @@
         <v>10000</v>
       </c>
       <c r="D10">
-        <f>B10-C10</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E10">
@@ -705,7 +814,7 @@
         <v>10000</v>
       </c>
       <c r="D11">
-        <f>B11-C11</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E11">
@@ -724,7 +833,7 @@
         <v>10000</v>
       </c>
       <c r="D12">
-        <f>B12-C12</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E12">
@@ -743,7 +852,7 @@
         <v>10000</v>
       </c>
       <c r="D13">
-        <f>B13-C13</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E13">
@@ -762,7 +871,7 @@
         <v>10000</v>
       </c>
       <c r="D14">
-        <f>B14-C14</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E14">
@@ -781,7 +890,7 @@
         <v>10000</v>
       </c>
       <c r="D15">
-        <f>B15-C15</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E15">
@@ -800,7 +909,7 @@
         <v>10000</v>
       </c>
       <c r="D16">
-        <f>B16-C16</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E16">
@@ -819,7 +928,7 @@
         <v>10000</v>
       </c>
       <c r="D17">
-        <f>B17-C17</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E17">
@@ -838,7 +947,7 @@
         <v>10000</v>
       </c>
       <c r="D18">
-        <f>B18-C18</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E18">
@@ -857,7 +966,7 @@
         <v>10000</v>
       </c>
       <c r="D19">
-        <f>B19-C19</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E19">
@@ -876,7 +985,7 @@
         <v>10000</v>
       </c>
       <c r="D20">
-        <f>B20-C20</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E20">
@@ -895,7 +1004,7 @@
         <v>10000</v>
       </c>
       <c r="D21">
-        <f>B21-C21</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E21">
@@ -914,7 +1023,7 @@
         <v>10000</v>
       </c>
       <c r="D22">
-        <f>B22-C22</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="E22">
@@ -935,16 +1044,16 @@
       <c r="A25" t="s">
         <v>17</v>
       </c>
-      <c r="B25" s="4" t="e">
-        <f>NPV([1]Assumptions!B2,D3:D22)+D2</f>
-        <v>#REF!</v>
+      <c r="B25" s="5">
+        <f>NPV(Assunzioni!B2,D3:D22)+D2</f>
+        <v>188195.27311391488</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>15</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="4">
         <f>(SUM(B2:B22)-SUM(C2:C22))/SUM(C2:C22)</f>
         <v>1</v>
       </c>
@@ -954,7 +1063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15F5DE18-B320-4E07-A514-5449D45B0C60}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -976,7 +1085,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1CE410-6A17-4169-858C-950C42088566}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1010,7 +1119,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8420DE59-92DF-4BC6-83EA-350D88661719}">
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1036,7 +1145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E4DE8D8-3DA8-4B13-87F1-B07DD665EB4F}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
[DASHBOARD] Add automatic cashflow and IRR charts
</commit_message>
<xml_diff>
--- a/models/financial/financial_model_crowdfunding.xlsx
+++ b/models/financial/financial_model_crowdfunding.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AdelinePruvost\Documents\circular-energy-fund\models\financial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91F4C12-D612-43AA-9BA8-A042E68E850B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9938A654-D96E-4776-9044-45834D241EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="240" windowWidth="17280" windowHeight="8880" xr2:uid="{D264A57A-F8FE-4DF8-A1A7-B185DC2A0E30}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>Fonte</t>
   </si>
@@ -113,7 +113,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-[$€-2]\ * #,##0.00_-;\-[$€-2]\ * #,##0.00_-;_-[$€-2]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -140,6 +140,13 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="22"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -187,18 +194,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -215,6 +224,3426 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Cashflow cumulato nel tempo</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-500000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-440000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-380000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-320000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-260000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-200000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-140000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="7"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-80000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="8"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>-20000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="9"/>
+          <c:order val="9"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>9</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000009-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="10"/>
+          <c:order val="10"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>100000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000A-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="11"/>
+          <c:order val="11"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>160000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000B-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="12"/>
+          <c:order val="12"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>220000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000C-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="13"/>
+          <c:order val="13"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>13</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>280000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000D-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="14"/>
+          <c:order val="14"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$16</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>340000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000E-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="15"/>
+          <c:order val="15"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$17</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>15</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$17</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>400000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000F-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="16"/>
+          <c:order val="16"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$18</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>460000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000010-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="17"/>
+          <c:order val="17"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$19</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>17</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>520000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000011-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="18"/>
+          <c:order val="18"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$20</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>580000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000012-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="19"/>
+          <c:order val="19"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$21</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>19</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>640000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000013-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="20"/>
+          <c:order val="20"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$22</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>700000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000014-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="21"/>
+          <c:order val="21"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$23</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000015-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="22"/>
+          <c:order val="22"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$24</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>IRR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000016-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="23"/>
+          <c:order val="23"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$25</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>NPV</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000017-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="24"/>
+          <c:order val="24"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$26</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ROI</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
+                    <a:lumOff val="40000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Cashflow!$E$26</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000018-0F8D-4A9D-8C3C-CA0ACCC9AA0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="215250127"/>
+        <c:axId val="215252047"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="215250127"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Anno</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="215252047"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="215252047"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>€</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="215250127"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>IRR progetto</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>IRR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$B$10</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.10315614602932954</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-7865-4D46-A689-76AB701775F1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="215263087"/>
+        <c:axId val="215263567"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="215263087"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="215263567"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="215263567"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="0.2"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="215263087"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>635000</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>78740</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>241300</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E44F0D9-5197-E518-DF28-480CF449892C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>78740</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>58420</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7FABC060-2645-5507-60D1-DEFDEA5AC23A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -534,7 +3963,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33298941-3A45-4CC1-A16E-D377190500EE}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
@@ -542,57 +3971,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="7">
         <f>Cashflow!B24</f>
         <v>0.10315614602932954</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="8">
         <f>Cashflow!B25</f>
         <v>188195.27311391488</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="7">
         <f>Cashflow!B26</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="8">
         <f>SUM(CAPEX!B:B)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="8">
         <f>MAX(Cashflow!E:E)</f>
         <v>700000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="12">
+        <f>Cashflow!B24</f>
+        <v>0.10315614602932954</v>
       </c>
     </row>
   </sheetData>
@@ -600,6 +4038,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
[DASHBOARD] Add break-even chart (cashflow cumulative)
</commit_message>
<xml_diff>
--- a/models/financial/financial_model_crowdfunding.xlsx
+++ b/models/financial/financial_model_crowdfunding.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AdelinePruvost\Documents\circular-energy-fund\models\financial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9938A654-D96E-4776-9044-45834D241EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F352D4B1-C933-4540-9E19-4FF895D2FD6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="240" windowWidth="17280" windowHeight="8880" xr2:uid="{D264A57A-F8FE-4DF8-A1A7-B185DC2A0E30}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>Fonte</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>Cashflow Finale</t>
+  </si>
+  <si>
+    <t>Linea Zero</t>
   </si>
 </sst>
 </file>
@@ -204,10 +207,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2457,6 +2460,2004 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Break-even – Cashflow cumulato</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$2,Cashflow!$F$2)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-500000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="sq">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:prstDash val="dot"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525" cap="sq">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:prstDash val="dot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$3,Cashflow!$F$3)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-440000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$4,Cashflow!$F$4)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-380000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$5,Cashflow!$F$5)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-320000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$6,Cashflow!$F$6)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-260000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$7,Cashflow!$F$7)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-200000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$8,Cashflow!$F$8)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-140000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="7"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$9,Cashflow!$F$9)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-80000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="8"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$10,Cashflow!$F$10)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>-20000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="9"/>
+          <c:order val="9"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>9</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$11,Cashflow!$F$11)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>40000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000009-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="10"/>
+          <c:order val="10"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$12,Cashflow!$F$12)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>100000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000A-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="11"/>
+          <c:order val="11"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$13,Cashflow!$F$13)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>160000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000B-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="12"/>
+          <c:order val="12"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$14,Cashflow!$F$14)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>220000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000C-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="13"/>
+          <c:order val="13"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>13</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$15,Cashflow!$F$15)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>280000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000D-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="14"/>
+          <c:order val="14"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$16</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$16,Cashflow!$F$16)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>340000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000E-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="15"/>
+          <c:order val="15"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$17</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>15</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$17,Cashflow!$F$17)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>400000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000F-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="16"/>
+          <c:order val="16"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$18</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$18,Cashflow!$F$18)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>460000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000010-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="17"/>
+          <c:order val="17"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$19</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>17</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$19,Cashflow!$F$19)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>520000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000011-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="18"/>
+          <c:order val="18"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$20</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$20,Cashflow!$F$20)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>580000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000012-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="19"/>
+          <c:order val="19"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$21</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>19</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$21,Cashflow!$F$21)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>640000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000013-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="20"/>
+          <c:order val="20"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$22</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$22,Cashflow!$F$22)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>700000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000014-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="21"/>
+          <c:order val="21"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$23</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$23,Cashflow!$F$23)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000015-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="22"/>
+          <c:order val="22"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$24</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>IRR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$24,Cashflow!$F$24)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000016-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="23"/>
+          <c:order val="23"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$25</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>NPV</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="80000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$25,Cashflow!$F$25)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000017-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="24"/>
+          <c:order val="24"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Cashflow!$A$26</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ROI</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
+                    <a:lumOff val="40000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>(Cashflow!$E$26,Cashflow!$F$26)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000018-A6A5-4EE0-84E3-85710D62C0C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="127464687"/>
+        <c:axId val="127463727"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="127464687"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Anno</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="127463727"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="127463727"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>€</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="127464687"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2537,6 +4538,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3054,6 +5095,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3638,6 +6195,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>635000</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>33020</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>393700</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8AD190C8-EC1D-B87A-4441-5DAAB3185EA0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3971,13 +6564,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -4025,10 +6618,10 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="10">
         <f>Cashflow!B24</f>
         <v>0.10315614602932954</v>
       </c>
@@ -4044,7 +6637,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E55BE27-92FE-47F5-9B77-15FAB5E6A743}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
@@ -4054,7 +6647,7 @@
     <col min="5" max="5" width="8.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -4070,8 +6663,11 @@
       <c r="E1" t="s">
         <v>14</v>
       </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -4089,8 +6685,11 @@
         <f>SUM(D$2:D2)</f>
         <v>-500000</v>
       </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4108,8 +6707,11 @@
         <f>SUM(D$2:D3)</f>
         <v>-440000</v>
       </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4127,8 +6729,11 @@
         <f>SUM(D$2:D4)</f>
         <v>-380000</v>
       </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -4146,8 +6751,11 @@
         <f>SUM(D$2:D5)</f>
         <v>-320000</v>
       </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -4165,8 +6773,11 @@
         <f>SUM(D$2:D6)</f>
         <v>-260000</v>
       </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -4184,8 +6795,11 @@
         <f>SUM(D$2:D7)</f>
         <v>-200000</v>
       </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -4203,8 +6817,11 @@
         <f>SUM(D$2:D8)</f>
         <v>-140000</v>
       </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -4222,8 +6839,11 @@
         <f>SUM(D$2:D9)</f>
         <v>-80000</v>
       </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -4241,8 +6861,11 @@
         <f>SUM(D$2:D10)</f>
         <v>-20000</v>
       </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -4260,8 +6883,11 @@
         <f>SUM(D$2:D11)</f>
         <v>40000</v>
       </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -4279,8 +6905,11 @@
         <f>SUM(D$2:D12)</f>
         <v>100000</v>
       </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -4298,8 +6927,11 @@
         <f>SUM(D$2:D13)</f>
         <v>160000</v>
       </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -4317,8 +6949,11 @@
         <f>SUM(D$2:D14)</f>
         <v>220000</v>
       </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -4336,8 +6971,11 @@
         <f>SUM(D$2:D15)</f>
         <v>280000</v>
       </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -4355,8 +6993,11 @@
         <f>SUM(D$2:D16)</f>
         <v>340000</v>
       </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
@@ -4374,8 +7015,11 @@
         <f>SUM(D$2:D17)</f>
         <v>400000</v>
       </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -4393,8 +7037,11 @@
         <f>SUM(D$2:D18)</f>
         <v>460000</v>
       </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
@@ -4412,8 +7059,11 @@
         <f>SUM(D$2:D19)</f>
         <v>520000</v>
       </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
@@ -4431,8 +7081,11 @@
         <f>SUM(D$2:D20)</f>
         <v>580000</v>
       </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
@@ -4450,8 +7103,11 @@
         <f>SUM(D$2:D21)</f>
         <v>640000</v>
       </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
@@ -4469,8 +7125,16 @@
         <f>SUM(D$2:D22)</f>
         <v>700000</v>
       </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>16</v>
       </c>
@@ -4478,8 +7142,11 @@
         <f>IRR(D2:D22)</f>
         <v>0.10315614602932954</v>
       </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -4487,14 +7154,20 @@
         <f>NPV(Assunzioni!B2,D3:D22)+D2</f>
         <v>188195.27311391488</v>
       </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>15</v>
       </c>
       <c r="B26" s="4">
         <f>(SUM(B2:B22)-SUM(C2:C22))/SUM(C2:C22)</f>
         <v>1</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>